<commit_message>
feat: add  pbstu with cfgtool  and  opt restApi
</commit_message>
<xml_diff>
--- a/tools/cfgtool/xls/Texas.xlsx
+++ b/tools/cfgtool/xls/Texas.xlsx
@@ -8,9 +8,8 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkCode\tools\bf_xlsx_tool\xls\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{979077A6-B3B3-4336-BCEB-BD3797679B2E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12255" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12255" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="德州扑克表" sheetId="1" r:id="rId1"/>
@@ -77,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="89">
   <si>
     <t>RoomStage</t>
   </si>
@@ -336,81 +335,96 @@
   <si>
     <t>31.12,44.111|978.012,7876.73;31.12,44.111|978.012,7876.73</t>
     <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>200|200|200|400|400</t>
+  </si>
+  <si>
+    <t>400|400|400|800|800</t>
+  </si>
+  <si>
+    <t>1000|1000|1000|2000|2000</t>
+  </si>
+  <si>
+    <t>A1|J3|K1;21|31</t>
+  </si>
+  <si>
+    <t>31.12|44.111;978.012|7876.73^31.12|44.111;978.012|7876.73</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <fonts count="10">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
+      <color theme="1"/>
+      <sz val="10"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
       <name val="微软雅黑"/>
       <charset val="134"/>
+      <color rgb="FF000000"/>
+      <sz val="9"/>
     </font>
     <font>
-      <sz val="9"/>
       <name val="宋体"/>
       <charset val="134"/>
+      <sz val="9"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
       <name val="宋体"/>
       <charset val="134"/>
+      <b val="1"/>
+      <sz val="9"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
       <sz val="9"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
       <sz val="9"/>
-      <color rgb="FF000000"/>
-      <name val="微软雅黑"/>
-      <family val="2"/>
-      <charset val="134"/>
     </font>
     <font>
-      <b/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -423,7 +437,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
+        <fgColor theme="7" tint="0.3999755851924192"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -444,16 +458,16 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color auto="true"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color auto="true"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color auto="true"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color auto="true"/>
       </bottom>
       <diagonal/>
     </border>
@@ -482,37 +496,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="true" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -520,7 +534,7 @@
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -533,7 +547,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="WPS">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WPS">
   <a:themeElements>
     <a:clrScheme name="WPS">
       <a:dk1>
@@ -783,22 +797,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M28"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="2" width="15.5" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.25" style="1" customWidth="1"/>
-    <col min="6" max="6" width="15.375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="14" style="1" customWidth="1"/>
-    <col min="8" max="8" width="15.625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5" style="1" customWidth="1"/>
-    <col min="10" max="10" width="30.375" style="4" customWidth="1"/>
-    <col min="11" max="12" width="17.25" style="1" customWidth="1"/>
-    <col min="13" max="13" width="35.125" style="1" customWidth="1"/>
+    <col customWidth="true" max="2" min="1" style="1" width="15.5"/>
+    <col customWidth="true" max="3" min="3" style="1" width="16.125"/>
+    <col customWidth="true" max="4" min="4" style="1" width="14"/>
+    <col customWidth="true" max="5" min="5" style="1" width="12.25"/>
+    <col customWidth="true" max="6" min="6" style="1" width="15.375"/>
+    <col customWidth="true" max="7" min="7" style="1" width="14"/>
+    <col customWidth="true" max="8" min="8" style="1" width="15.625"/>
+    <col customWidth="true" max="9" min="9" style="1" width="14.5"/>
+    <col customWidth="true" max="10" min="10" style="4" width="30.375"/>
+    <col customWidth="true" max="12" min="11" style="1" width="17.25"/>
+    <col customWidth="true" max="13" min="13" style="1" width="35.125"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:13" ht="14.25">
       <c r="A1" s="3" t="s">
         <v>18</v>
       </c>
@@ -839,7 +853,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:13" ht="14.25">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -880,7 +894,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:13" ht="14.25">
       <c r="A3" s="3" t="s">
         <v>13</v>
       </c>
@@ -921,7 +935,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="14.25" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:13" ht="14.25">
       <c r="A4" s="7" t="s">
         <v>77</v>
       </c>
@@ -962,7 +976,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:13">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -991,7 +1005,7 @@
         <v>6</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>31</v>
+        <v>84</v>
       </c>
       <c r="K5" s="1">
         <v>100</v>
@@ -1003,7 +1017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:13">
       <c r="A6" s="1">
         <v>2</v>
       </c>
@@ -1032,7 +1046,7 @@
         <v>6</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
       <c r="K6" s="1">
         <v>100</v>
@@ -1044,7 +1058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:13">
       <c r="A7" s="1">
         <v>3</v>
       </c>
@@ -1073,7 +1087,7 @@
         <v>6</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>33</v>
+        <v>86</v>
       </c>
       <c r="K7" s="1">
         <v>100</v>
@@ -1085,7 +1099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:13">
       <c r="A8" s="1">
         <v>1</v>
       </c>
@@ -1114,7 +1128,7 @@
         <v>6</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>31</v>
+        <v>84</v>
       </c>
       <c r="K8" s="1">
         <v>100</v>
@@ -1126,7 +1140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:13">
       <c r="A9" s="1">
         <v>2</v>
       </c>
@@ -1155,7 +1169,7 @@
         <v>6</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
       <c r="K9" s="1">
         <v>100</v>
@@ -1167,7 +1181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:13">
       <c r="A10" s="1">
         <v>3</v>
       </c>
@@ -1196,7 +1210,7 @@
         <v>6</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>33</v>
+        <v>86</v>
       </c>
       <c r="K10" s="1">
         <v>100</v>
@@ -1208,28 +1222,40 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="13:13" x14ac:dyDescent="0.15">
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23" spans="13:13">
       <c r="M23" s="6"/>
     </row>
-    <row r="24" spans="13:13" x14ac:dyDescent="0.15">
+    <row r="24" spans="13:13">
       <c r="M24" s="6"/>
     </row>
-    <row r="25" spans="13:13" x14ac:dyDescent="0.15">
+    <row r="25" spans="13:13">
       <c r="M25" s="6"/>
     </row>
-    <row r="26" spans="13:13" x14ac:dyDescent="0.15">
+    <row r="26" spans="13:13">
       <c r="M26" s="4"/>
     </row>
-    <row r="27" spans="13:13" x14ac:dyDescent="0.15">
+    <row r="27" spans="13:13">
       <c r="M27" s="4"/>
     </row>
-    <row r="28" spans="13:13" x14ac:dyDescent="0.15">
+    <row r="28" spans="13:13">
       <c r="M28" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup r:id="rId1" orientation="portrait" paperSize="9"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -1479,17 +1505,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:L8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="13" style="1" customWidth="1"/>
-    <col min="2" max="2" width="16.125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="70.25" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10" style="1" customWidth="1"/>
-    <col min="5" max="5" width="9.75" style="1" customWidth="1"/>
-    <col min="6" max="12" width="10.25" customWidth="1"/>
+    <col customWidth="true" max="1" min="1" style="1" width="13"/>
+    <col customWidth="true" max="2" min="2" style="1" width="16.125"/>
+    <col customWidth="true" max="3" min="3" style="1" width="70.25"/>
+    <col customWidth="true" max="4" min="4" style="1" width="10"/>
+    <col customWidth="true" max="5" min="5" style="1" width="9.75"/>
+    <col customWidth="true" max="12" min="6" width="10.25"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:12">
       <c r="A1" s="2" t="s">
         <v>63</v>
       </c>
@@ -1527,7 +1553,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:12">
       <c r="A2" s="2" t="s">
         <v>50</v>
       </c>
@@ -1565,7 +1591,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:12">
       <c r="A3" s="2" t="s">
         <v>15</v>
       </c>
@@ -1603,7 +1629,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:12">
       <c r="A4" s="8" t="s">
         <v>78</v>
       </c>
@@ -1641,15 +1667,15 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:12">
       <c r="A5" s="1">
         <v>1</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>66</v>
@@ -1679,15 +1705,15 @@
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:12">
       <c r="A6" s="1">
         <v>2</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>66</v>
@@ -1717,15 +1743,15 @@
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:12">
       <c r="A7" s="1">
         <v>3</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>66</v>
@@ -1755,15 +1781,15 @@
         <v>71</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:12">
       <c r="A8" s="1">
         <v>4</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>66</v>
@@ -1796,7 +1822,7 @@
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup r:id="rId1" orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
 

</xml_diff>